<commit_message>
feat: Azure-style diagram coloring, release-over-release diffs, L0/L1 nav integration
- Platform arch diagrams: color-coded lanes (blue=cloud, purple=SaaS, green=on-prem, teal=data, orange=middleware)
- Data arch diagrams: DB cylinders colored by category (cloud/data-platform/on-prem)
- Color legends added to both diagram types
- New section 5.3 Release-over-Release Changes in L0/L1/Program summaries
  - Auto-discovers R1/R2/R3 release data per capability
  - Shows app/DB/platform additions and retirements between releases
- L0/L1 summary links in all 3 sidebar JS instances + tower hero + index hero
- nav.json now includes l0_summary and l1_summary fields
- Backfilled DS-020 flow data (47 columns, R1-R3)
- Data architecture redesign: DB-to-DB flows instead of entity-centric
- Fixed Unicode encoding issues in gen_tower_pages.py print statements
</commit_message>
<xml_diff>
--- a/towers/FPR/DS Provide Decision Support/DS-020/input/data/CurrentFlows.xlsx
+++ b/towers/FPR/DS Provide Decision Support/DS-020/input/data/CurrentFlows.xlsx
@@ -878,6 +878,116 @@
           <t>https://iapm.intel.com/#/app/35612</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>MES 300 → XEUS: MES Routes</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Kerberos / X.509</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>IF-MESRouteto-01</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>MES300_PROD.MES_Routes</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>XEUS_PROD.MES_Routes</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Intel MES On-Premise</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Intel Middleware On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -985,6 +1095,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>XEUS → ICOST: FSM/ATM SF Routes &amp; Cycle Times</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>JMS / File</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>IF-MESRouteto-02</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>XEUS_PROD.FSM_ATM_SF_Routes_&amp;_Cycle_Time</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.FSM_ATM_SF_Routes_&amp;_Cycle_Time</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>Intel Middleware On-Premise</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1097,6 +1317,116 @@
           <t>https://iapm.intel.com/#/app/33537</t>
         </is>
       </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Forecast Data</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>CSV / JSON</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>WorkStream → MARS: WorkStream Routes</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>IF-WorkStream-01</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>WS_PROD.WorkStream_Routes</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>MARS_PROD.WorkStream_Routes</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>Intel MES On-Premise</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1204,6 +1534,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>MARS → ICOST: Forecast ASP / Forecast Units</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>IF-WSForecast-02</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>MARS_PROD.Forecast_ASP___Forecast_Units</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.Forecast_ASP___Forecast_Units</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1301,6 +1741,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>EATS → ICOST: ATM Cycle Times</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>IF-ATMCycleTi-01</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>EATS_PROD.ATM_Cycle_Times</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.ATM_Cycle_Times</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1414,6 +1964,116 @@
           <t>https://iapm.intel.com/#/app/21195</t>
         </is>
       </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Material Master</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>SPEED → SAP PO: Material Master &amp; BOMs</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>IF-SPEEDBOMto-01</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>SPEED_PROD.Material_Master_&amp;_BOMs</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>SAPPO.Material_Master_&amp;_BOMs</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1516,6 +2176,116 @@
           <t>https://iapm.intel.com/#/app/23736</t>
         </is>
       </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>SAP PO → SAP ECC: Material BOMs, RM Std Cost, RM Inv</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>RFC / SOAP / IDoc</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>X.509 / Basic Auth</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>IF-SPEEDBOMto-02</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>SAPPO.Material_BOMs,_RM_Std_Cost,_RM</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>SAPSR3.Material_BOMs,_RM_Std_Cost,_RM</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1627,6 +2397,116 @@
       <c r="Y9" t="inlineStr">
         <is>
           <t>https://iapm.intel.com/#/app/4010</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Bill of Materials</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>SPEED → EDW: Product BOMs</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>REST / File</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>IF-SPEEDBOMto-01</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>SPEED_PROD.Product_BOMs</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>EDW_PROD.Product_BOMs</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
         </is>
       </c>
     </row>
@@ -1738,6 +2618,116 @@
           <t>https://iapm.intel.com/#/app/23736</t>
         </is>
       </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Legacy MDG → SAP ECC: Master Data</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>SAP SSO</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>IF-MasterData-01</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>SAPSR3.Master_Data</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>SAPSR3.Master_Data</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>SAP ECC MDG On-Premise</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1835,6 +2825,116 @@
           <t>https://iapm.intel.com/#/app/21195</t>
         </is>
       </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Material Master</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>CIBR → SAP PO: RM Inv Consumption &amp; Subcon Inv Data</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>IF-CIBRRMInvt-01</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>CIBR_PROD.RM_Inv_Consumption_&amp;_Subcon_In</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>SAPPO.RM_Inv_Consumption_&amp;_Subcon_In</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1932,6 +3032,116 @@
           <t>https://iapm.intel.com/#/app/23736</t>
         </is>
       </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>SAP PO → SAP ECC: RM Inv Consumption &amp; Subcon Inv Data</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>RFC / SOAP / IDoc</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>X.509 / Basic Auth</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>IF-CIBRRMInvt-02</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>SAPPO.RM_Inv_Consumption_&amp;_Subcon_In</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>SAPSR3.RM_Inv_Consumption_&amp;_Subcon_In</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2034,6 +3244,116 @@
           <t>https://iapm.intel.com/#/app/42993</t>
         </is>
       </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Bill of Materials</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>SAP ECC → SideCar: SLT: Financials, BOMs, Routes</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>IF-ECCReplica-01</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>SAPSR3.SLT:_Financials,_BOMs,_Routes</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>SIDECAR_DB.SLT:_Financials,_BOMs,_Routes</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2136,6 +3456,116 @@
           <t>https://iapm.intel.com/#/app/25794</t>
         </is>
       </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>SideCar → Azure ADF: CIF Data</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>HANA SQL / SDA</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>SAP SSO</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>IF-ECCReplica-02</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>N/A (ETL)</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>SIDECAR_DB.CIF_Data</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>Azure Data Factory Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2233,6 +3663,116 @@
           <t>https://iapm.intel.com/#/app/41458</t>
         </is>
       </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Azure ADF → DataBricks: Transform Data</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>REST / JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Azure AD / Managed Identity</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>IF-ECCReplica-03</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>N/A (ETL)</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>Delta Lake</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>unity_catalog.Transform_Data</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Azure Data Factory Cloud</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>Databricks Cloud SaaS</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2341,6 +3881,116 @@
           <t>https://iapm.intel.com/#/app/35811</t>
         </is>
       </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>DataBricks → SnowFlake: Stores Data</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>SQL / REST / Spark</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Azure AD / PAT</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>IF-ECCReplica-04</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Delta Lake</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Snowflake Cloud DW</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>unity_catalog.Stores_Data</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>INTEL_DW.Stores_Data</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Databricks Cloud SaaS</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Snowflake Cloud SaaS</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2448,6 +4098,116 @@
           <t>https://iapm.intel.com/#/app/43119</t>
         </is>
       </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Corp / IP S/4 → ECA: Inv Mvt Conf (561 MvT) BOH Transfer</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>RFC / OData</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>SAP SSO / X.509</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>IF-Corp/IPInv-01</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>Azure Data Lake (ADLS)</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>SAPHANADB.Inv_Mvt_Conf_(561_MvT)_BOH_Tra</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>ECA_LAKE.Inv_Mvt_Conf_(561_MvT)_BOH_Tra</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA On-Premise</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>Intel ECA Platform Azure Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2555,6 +4315,116 @@
           <t>https://iapm.intel.com/#/app/43119</t>
         </is>
       </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Material Master</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>Corp / IP S/4 → ECA: Master data: Finance, Materials (BOM), Plant Calendar</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>RFC / OData</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>SAP SSO / X.509</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>IF-Corp/IPMas-01</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>Azure Data Lake (ADLS)</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>SAPHANADB.Master_data:_Finance,_Material</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>ECA_LAKE.Master_data:_Finance,_Material</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA On-Premise</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>Intel ECA Platform Azure Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2662,6 +4532,116 @@
           <t>https://iapm.intel.com/#/app/237</t>
         </is>
       </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>ECA → CIBR: Inv Mvt Conf (ECA to CIBR)</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>REST / Spark SQL</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>Azure AD / Service Principal</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>IF-ECACosting-01</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Azure Data Lake (ADLS)</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>ECA_LAKE.Inv_Mvt_Conf_(ECA_to_CIBR)</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>CIBR_PROD.Inv_Mvt_Conf_(ECA_to_CIBR)</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>Intel ECA Platform Azure Cloud</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2764,6 +4744,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>CIBR → ICOST: WIP &amp; FG</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>IF-ECACosting-02</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>CIBR_PROD.WIP_&amp;_FG</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.WIP_&amp;_FG</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2871,6 +4961,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>ECA → ICOST: Cost Data</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>REST / Spark SQL</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>Azure AD / Service Principal</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>IF-ECACosting-03</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>Azure Data Lake (ADLS)</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>ECA_LAKE.Cost_Data</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.Cost_Data</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>Intel ECA Platform Azure Cloud</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2973,6 +5173,116 @@
           <t>https://iapm.intel.com/#/app/19207</t>
         </is>
       </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>ICOST → SAP BODS: GL Postings</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>NTLM / Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>IF-GLPostingt-01</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.GL_Postings</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>BODS_REPO.GL_Postings</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>SAP Data Services On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3075,6 +5385,116 @@
           <t>https://iapm.intel.com/#/app/23736</t>
         </is>
       </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>GL Account</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>BAPI / OData</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>SAP BODS → SAP ECC: GL Postings</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>JDBC / File / RFC</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>OS Auth / DB Auth</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>IF-GLPostingt-02</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>BODS_REPO.GL_Postings</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>SAPSR3.GL_Postings</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>SAP Data Services On-Premise</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3182,6 +5602,116 @@
           <t>https://iapm.intel.com/#/app/41052</t>
         </is>
       </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>GL Account</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>BAPI / OData</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>SAP ECC → CFIN S/4: Replicated GL Postings</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>IF-GLPostingt-03</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>SAPSR3.Replicated_GL_Postings</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>SAPHANADB.Replicated_GL_Postings</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Central Finance</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3279,6 +5809,116 @@
           <t>https://iapm.intel.com/#/app/4010</t>
         </is>
       </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Material Master</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>IDoc / CSV</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>Intel Restricted</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>SAP ECC → EDW: Finance Master Data, G/L Spending, BOM, Materials, Order Details</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>IF-ECCtoEDWRe-01</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>SAPSR3.Finance_Master_Data,_G_L_Spend</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>EDW_PROD.Finance_Master_Data,_G_L_Spend</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3376,6 +6016,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>EDW → ICOST: Inventory Data, Cost Data, GL Transactions</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>LDAP / Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>IF-EDWFeedbac-01</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>EDW_PROD.Inventory_Data,_Cost_Data,_GL_</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.Inventory_Data,_Cost_Data,_GL_</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3473,6 +6223,116 @@
           <t>https://iapm.intel.com/#/app/237</t>
         </is>
       </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>EDW → CIBR: Cost &amp; Inventory Data</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>LDAP / Kerberos</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>IF-EDWFeedbac-01</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>EDW_PROD.Cost_&amp;_Inventory_Data</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>CIBR_PROD.Cost_&amp;_Inventory_Data</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3570,6 +6430,116 @@
           <t>https://iapm.intel.com/#/app/9008</t>
         </is>
       </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>FCA → ICOST: Financial Cost Data</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>JDBC / File</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>Kerberos / NTLM</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>IF-FCAtoICOST-01</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>FCA_PROD.Financial_Cost_Data</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>ICOST_PROD.Financial_Cost_Data</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>Intel Custom On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3672,6 +6642,116 @@
           <t>https://iapm.intel.com/#/app/42993</t>
         </is>
       </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>SAP ECC → Finance HANA: Finance Data</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>&lt; 1 second (real-time)</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>IF-ECCtoFinan-01</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ29" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>SAPSR3.Finance_Data</t>
+        </is>
+      </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>FINANCE_DB.Finance_Data</t>
+        </is>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3779,6 +6859,116 @@
           <t>https://iapm.intel.com/#/app/22790</t>
         </is>
       </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>Finance HANA → APIGEE: RM Std Major Fluctuations</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>HANA SQL / SDA</t>
+        </is>
+      </c>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>SAP SSO / X.509</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>IF-RMStdFluct-01</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN30" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO30" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP30" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ30" t="inlineStr">
+        <is>
+          <t>N/A (API Gateway)</t>
+        </is>
+      </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>FINANCE_DB.RM_Std_Major_Fluctuations</t>
+        </is>
+      </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>Google Apigee Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3886,6 +7076,116 @@
           <t>https://iapm.intel.com/#/app/43163</t>
         </is>
       </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>APIGEE → PEGA: RM Std Major Fluctuations</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>REST / GraphQL</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>OAuth 2.0 / API Key</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>IF-RMStdFluct-02</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>N/A (API Gateway)</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>PEGA_PROD.RM_Std_Major_Fluctuations</t>
+        </is>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t>Google Apigee Cloud</t>
+        </is>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>Pega Cloud SaaS</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3978,6 +7278,116 @@
           <t>https://iapm.intel.com/#/app/17651</t>
         </is>
       </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Financial Report</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>CSV / PDF</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>Finance HANA → BOBJ: Financial Analytics Data</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>HANA SQL / SDA</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>SAP SSO / X.509</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>IF-FinanceHAN-01</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>FINANCE_DB.Financial_Analytics_Data</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>BOBJ_CMS.Financial_Analytics_Data</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>SAP BusinessObjects On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4075,6 +7485,116 @@
           <t>https://iapm.intel.com/#/app/21195</t>
         </is>
       </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>Finance HANA → SAP PO: RM Std Cost Update</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>HANA SQL / SDA</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>SAP SSO / X.509</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>IF-RMStdCostU-01</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>SAP HANA</t>
+        </is>
+      </c>
+      <c r="AQ33" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>FINANCE_DB.RM_Std_Cost_Update</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>SAPPO.RM_Std_Cost_Update</t>
+        </is>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>SAP HANA Sidecar On-Premise</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4172,6 +7692,116 @@
           <t>https://iapm.intel.com/#/app/23736</t>
         </is>
       </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Cost Element</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>IDoc / Flat File</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>SAP PO → SAP ECC: RM Std Cost Update</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>Direct / SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>RFC / SOAP / IDoc</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>X.509 / Basic Auth</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>IF-RMStdCostU-02</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>SAPPO.RM_Std_Cost_Update</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>SAPSR3.RM_Std_Cost_Update</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>SAP Process Orchestration On-Premise</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4284,6 +7914,116 @@
           <t>https://iapm.intel.com/#/app/43119</t>
         </is>
       </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Plan Data</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>CSV / JSON</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>~10K events/hour</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>SAP IBP → ECA: LCM Reserves, Financial Projections</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>REST / OData / CPI</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>OAuth 2.0 / SAML</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>&lt; 1 hour (near real-time)</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>IF-IBPDemandP-01</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>Point-to-Point</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>SAP HANA Cloud</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr">
+        <is>
+          <t>Azure Data Lake (ADLS)</t>
+        </is>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>IBP_HANA.LCM_Reserves,_Financial_Projec</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>ECA_LAKE.LCM_Reserves,_Financial_Projec</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>SAP IBP Cloud SaaS</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>Intel ECA Platform Azure Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4381,6 +8121,116 @@
           <t>https://iapm.intel.com/#/app/4010</t>
         </is>
       </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>SAP ECC → EDW: G/L Spending</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK36" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>IF-ECCGLtoEDW-01</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO36" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP36" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ36" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR36" t="inlineStr">
+        <is>
+          <t>SAPSR3.G_L_Spending</t>
+        </is>
+      </c>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>EDW_PROD.G_L_Spending</t>
+        </is>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4476,6 +8326,116 @@
       <c r="Y37" t="inlineStr">
         <is>
           <t>https://iapm.intel.com/#/app/4010</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Business Data</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>JSON / CSV</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>Intel Confidential</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>~50K-500K records/day</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>SAP ECC → EDW: BOH Transfer 711 MvT</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>SAP CPI</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>RFC / IDoc</t>
+        </is>
+      </c>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>SAP SSO / SNC</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>DEV, QAS, PRD</t>
+        </is>
+      </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>&lt; 4 hours (batch window)</t>
+        </is>
+      </c>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>IF-ECCBOHtoED-01</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>ETL / Batch</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>Retry 3x → Dead Letter Queue → Alert</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>SAP CCMS / Azure Monitor / Splunk</t>
+        </is>
+      </c>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>Oracle DB</t>
+        </is>
+      </c>
+      <c r="AQ37" t="inlineStr">
+        <is>
+          <t>Teradata / Oracle DB</t>
+        </is>
+      </c>
+      <c r="AR37" t="inlineStr">
+        <is>
+          <t>SAPSR3.BOH_Transfer_711_MvT</t>
+        </is>
+      </c>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>EDW_PROD.BOH_Transfer_711_MvT</t>
+        </is>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>SAP ECC 6.0 On-Premise</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>Intel EDW On-Premise</t>
         </is>
       </c>
     </row>

</xml_diff>